<commit_message>
MACC runs enabled for TRA, POW
This commit include initial changes and updates to enable MACC runs on transport and power sectors
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_Par-ESB_scens.xlsx
+++ b/SuppXLS/Scen_Par-ESB_scens.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbsul\Documents\GitHub\times-ireland-model\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2BBD6AE-81B3-4430-9BF0-E42BA1776058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68BF2FA7-82AE-4802-9C2E-4C83E7DC3C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="25760" windowHeight="15440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="controller" sheetId="15" r:id="rId1"/>
@@ -5036,7 +5036,7 @@
         <v>22</v>
       </c>
       <c r="J8" s="9">
-        <v>7.4999999999999997E-2</v>
+        <v>0.04</v>
       </c>
       <c r="K8" t="s">
         <v>23</v>
@@ -5056,7 +5056,7 @@
         <v>22</v>
       </c>
       <c r="J9" s="9">
-        <v>7.4999999999999997E-2</v>
+        <v>0.04</v>
       </c>
       <c r="K9" t="s">
         <v>23</v>
@@ -5076,7 +5076,7 @@
         <v>22</v>
       </c>
       <c r="J10" s="9">
-        <v>0.13500000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="K10" t="s">
         <v>23</v>
@@ -5096,7 +5096,7 @@
         <v>22</v>
       </c>
       <c r="J11" s="9">
-        <v>7.4999999999999997E-2</v>
+        <v>0.04</v>
       </c>
       <c r="K11" t="s">
         <v>23</v>
@@ -5116,7 +5116,7 @@
         <v>22</v>
       </c>
       <c r="J12" s="9">
-        <v>9.5000000000000001E-2</v>
+        <v>0.04</v>
       </c>
       <c r="K12" t="s">
         <v>23</v>
@@ -5136,7 +5136,7 @@
         <v>22</v>
       </c>
       <c r="J13" s="9">
-        <v>0.11</v>
+        <v>0.04</v>
       </c>
       <c r="K13" t="s">
         <v>23</v>

</xml_diff>